<commit_message>
update data package at: 2026-09-14T06:58:42
</commit_message>
<xml_diff>
--- a/data/BASE_REPASSE_RECURSOS.xlsx
+++ b/data/BASE_REPASSE_RECURSOS.xlsx
@@ -493,7 +493,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>880513540</v>
+        <v>901779262</v>
       </c>
     </row>
     <row r="3">
@@ -625,7 +625,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1131169707</v>
+        <v>1186551659</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
update data package at: 2026-09-21T07:17:49
</commit_message>
<xml_diff>
--- a/data/BASE_REPASSE_RECURSOS.xlsx
+++ b/data/BASE_REPASSE_RECURSOS.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,68 +465,68 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>2071</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FUNDAÇÃO DE AMPARO À PESQUISA DO ESTADO DE MINAS GERAIS</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>4711</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>1031</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>TRIBUNAL DE JUSTIÇA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="G2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>901779262</v>
+        <v>18603</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4491</v>
+        <v>4711</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE CULTURA</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2201</v>
+        <v>1031</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>INSTITUTO ESTADUAL DO PATRIMÔNIO HISTÓRICO E ARTÍSTICO DE MINAS GERAIS</t>
+          <t>TRIBUNAL DE JUSTIÇA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1000</v>
+        <v>901779262</v>
       </c>
     </row>
     <row r="4">
@@ -539,11 +539,11 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2171</v>
+        <v>2201</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO DE ARTE DE OURO PRETO</t>
+          <t>INSTITUTO ESTADUAL DO PATRIMÔNIO HISTÓRICO E ARTÍSTICO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -572,11 +572,11 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2181</v>
+        <v>2171</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO CLÓVIS SALGADO</t>
+          <t>FUNDAÇÃO DE ARTE DE OURO PRETO</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -597,35 +597,35 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4711</v>
+        <v>4491</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO ESTADUAL DE CULTURA</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1031</v>
+        <v>2181</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TRIBUNAL DE JUSTIÇA DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDAÇÃO CLÓVIS SALGADO</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1186551659</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7">
@@ -638,18 +638,18 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1441</v>
+        <v>1031</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DEFENSORIA PUBLICA DO ESTADO DE MINAS GERAIS</t>
+          <t>TRIBUNAL DE JUSTIÇA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G7" t="n">
         <v>5</v>
@@ -658,7 +658,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>72184243</v>
+        <v>1186551659</v>
       </c>
     </row>
     <row r="8">
@@ -682,7 +682,7 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G8" t="n">
         <v>5</v>
@@ -691,73 +691,73 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>105515757</v>
+        <v>72184243</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2101</v>
+        <v>4711</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>INSTITUTO ESTADUAL DE FLORESTAS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1401</v>
+        <v>1441</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CORPO DE BOMBEIROS MILITAR DO ESTADO DE MINAS GERAIS</t>
+          <t>DEFENSORIA PUBLICA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>7016160</v>
+        <v>105515757</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4711</v>
+        <v>2101</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>INSTITUTO ESTADUAL DE FLORESTAS</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1091</v>
+        <v>1401</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PROCURADORIA GERAL DE JUSTIÇA</t>
+          <t>CORPO DE BOMBEIROS MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="G10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>300411652</v>
+        <v>7016160</v>
       </c>
     </row>
     <row r="11">
@@ -781,7 +781,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G11" t="n">
         <v>5</v>
@@ -790,73 +790,73 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>448050447</v>
+        <v>300411652</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>4381</v>
+        <v>4711</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1191</v>
+        <v>1091</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA</t>
+          <t>PROCURADORIA GERAL DE JUSTIÇA</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>83</v>
+        <v>42</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>1008000</v>
+        <v>448050447</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>4711</v>
+        <v>4381</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1021</v>
+        <v>1191</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>TRIBUNAL DE CONTAS DO ESTADO DE MINAS GERAIS</t>
+          <t>SECRETARIA DE ESTADO DE FAZENDA</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>43</v>
+        <v>83</v>
       </c>
       <c r="G13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>133292078</v>
+        <v>1008000</v>
       </c>
     </row>
     <row r="14">
@@ -880,7 +880,7 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G14" t="n">
         <v>5</v>
@@ -889,7 +889,7 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>115233552</v>
+        <v>133292078</v>
       </c>
     </row>
     <row r="15">
@@ -902,18 +902,18 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1051</v>
+        <v>1021</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>TRIBUNAL DE JUSTIÇA MILITAR DO ESTADO DE MINAS GERAIS</t>
+          <t>TRIBUNAL DE CONTAS DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G15" t="n">
         <v>5</v>
@@ -922,7 +922,7 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>8800648</v>
+        <v>115233552</v>
       </c>
     </row>
     <row r="16">
@@ -946,7 +946,7 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G16" t="n">
         <v>5</v>
@@ -955,7 +955,7 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>11045990</v>
+        <v>8800648</v>
       </c>
     </row>
     <row r="17">
@@ -968,18 +968,18 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1011</v>
+        <v>1051</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
+          <t>TRIBUNAL DE JUSTIÇA MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E17" t="n">
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G17" t="n">
         <v>5</v>
@@ -988,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>129510000</v>
+        <v>11045990</v>
       </c>
     </row>
     <row r="18">
@@ -1012,7 +1012,7 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G18" t="n">
         <v>5</v>
@@ -1021,64 +1021,64 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>120000000</v>
+        <v>129510000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2261</v>
+        <v>4711</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO EZEQUIEL DIAS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4711</v>
+        <v>1011</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E19" t="n">
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="G19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>34739894</v>
+        <v>120000000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1301</v>
+        <v>2261</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIAS</t>
+          <t>FUNDAÇÃO EZEQUIEL DIAS</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4631</v>
+        <v>4711</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>FUNDO DE PAGAMENTO DE PARCERIAS PÚBLICO - PRIVADAS DE MINAS GERAIS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -1087,31 +1087,31 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>727000</v>
+        <v>34739894</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>4381</v>
+        <v>1301</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIAS</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2471</v>
+        <v>4631</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AGÊNCIA REGULADORA DE TRANSPORTES DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO DE PAGAMENTO DE PARCERIAS PÚBLICO - PRIVADAS DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
@@ -1120,7 +1120,7 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>17964220</v>
+        <v>727000</v>
       </c>
     </row>
     <row r="22">
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
         <v>60</v>
@@ -1153,31 +1153,31 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>5780000</v>
+        <v>17964220</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2371</v>
+        <v>4381</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>INSTITUTO MINEIRO DE AGROPECUÁRIA</t>
+          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1501</v>
+        <v>2471</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>AGÊNCIA REGULADORA DE TRANSPORTES DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>3</v>
       </c>
       <c r="F23" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="G23" t="n">
         <v>2</v>
@@ -1186,31 +1186,31 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>149161</v>
+        <v>5780000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2091</v>
+        <v>2371</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
+          <t>INSTITUTO MINEIRO DE AGROPECUÁRIA</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>4711</v>
+        <v>1501</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G24" t="n">
         <v>2</v>
@@ -1219,28 +1219,28 @@
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>155090</v>
+        <v>149161</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2121</v>
+        <v>2091</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES MILITARES DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1401</v>
+        <v>4711</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CORPO DE BOMBEIROS MILITAR DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
         <v>60</v>
@@ -1252,7 +1252,7 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>575076</v>
+        <v>155090</v>
       </c>
     </row>
     <row r="26">
@@ -1273,7 +1273,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
         <v>60</v>
@@ -1285,7 +1285,7 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>1004919</v>
+        <v>575076</v>
       </c>
     </row>
     <row r="27">
@@ -1298,18 +1298,18 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1251</v>
+        <v>1401</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
+          <t>CORPO DE BOMBEIROS MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G27" t="n">
         <v>2</v>
@@ -1318,7 +1318,7 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>15642001</v>
+        <v>1004919</v>
       </c>
     </row>
     <row r="28">
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F28" t="n">
         <v>49</v>
@@ -1351,7 +1351,7 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>140778004</v>
+        <v>15642001</v>
       </c>
     </row>
     <row r="29">
@@ -1364,18 +1364,18 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1501</v>
+        <v>1251</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>3</v>
       </c>
       <c r="F29" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="G29" t="n">
         <v>2</v>
@@ -1384,16 +1384,16 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>107449</v>
+        <v>140778004</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2091</v>
+        <v>2121</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
+          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES MILITARES DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1408,7 +1408,7 @@
         <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="G30" t="n">
         <v>2</v>
@@ -1417,7 +1417,7 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>2177178</v>
+        <v>107449</v>
       </c>
     </row>
     <row r="31">
@@ -1430,18 +1430,18 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1371</v>
+        <v>1501</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE MEIO AMBIENTE E DESENVOLVIMENTO SUSTENTÁVEL</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E31" t="n">
         <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="G31" t="n">
         <v>2</v>
@@ -1450,31 +1450,31 @@
         <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>13650000</v>
+        <v>2177178</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2241</v>
+        <v>2091</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>INSTITUTO MINEIRO DE GESTÃO DAS ÁGUAS</t>
+          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1501</v>
+        <v>1371</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>SECRETARIA DE ESTADO DE MEIO AMBIENTE E DESENVOLVIMENTO SUSTENTÁVEL</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>91</v>
+        <v>52</v>
       </c>
       <c r="G32" t="n">
         <v>2</v>
@@ -1483,31 +1483,31 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>1774713</v>
+        <v>13650000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2041</v>
+        <v>2241</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>LOTERIA DO ESTADO DE MINAS GERAIS</t>
+          <t>INSTITUTO MINEIRO DE GESTÃO DAS ÁGUAS</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4711</v>
+        <v>1501</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G33" t="n">
         <v>2</v>
@@ -1516,7 +1516,7 @@
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>1686000</v>
+        <v>1774713</v>
       </c>
     </row>
     <row r="34">
@@ -1529,15 +1529,15 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1501</v>
+        <v>4711</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
         <v>60</v>
@@ -1549,16 +1549,16 @@
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>458582</v>
+        <v>1686000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2441</v>
+        <v>2041</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>AGÊNCIA REGULADORA DE SERVIÇOS DE ABASTECIMENTO DE ÁGUA E DE ESGOTAMENTO SANITÁRIO DO ESTADO DE MINAS GERAIS</t>
+          <t>LOTERIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1573,7 +1573,7 @@
         <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
@@ -1582,31 +1582,31 @@
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>1707737</v>
+        <v>458582</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2251</v>
+        <v>2441</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>JUNTA COMERCIAL DO ESTADO DE MINAS GERAIS</t>
+          <t>AGÊNCIA REGULADORA DE SERVIÇOS DE ABASTECIMENTO DE ÁGUA E DE ESGOTAMENTO SANITÁRIO DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>4711</v>
+        <v>1501</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G36" t="n">
         <v>2</v>
@@ -1615,16 +1615,16 @@
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>4444845</v>
+        <v>1707737</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2321</v>
+        <v>2251</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO CENTRO DE HEMATOLOGIA E HEMOTERAPIA DE MINAS GERAIS</t>
+          <t>JUNTA COMERCIAL DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1648,31 +1648,31 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>31836274</v>
+        <v>4444845</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>2101</v>
+        <v>2321</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>INSTITUTO ESTADUAL DE FLORESTAS</t>
+          <t>FUNDAÇÃO CENTRO DE HEMATOLOGIA E HEMOTERAPIA DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1501</v>
+        <v>4711</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="G38" t="n">
         <v>2</v>
@@ -1681,16 +1681,16 @@
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>3110043</v>
+        <v>31836274</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>4031</v>
+        <v>2101</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>FUNDO ESPECIAL DO PODER JUDICIÁRIO DO ESTADO DE MINAS GERAIS</t>
+          <t>INSTITUTO ESTADUAL DE FLORESTAS</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1705,7 +1705,7 @@
         <v>3</v>
       </c>
       <c r="F39" t="n">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G39" t="n">
         <v>2</v>
@@ -1714,7 +1714,7 @@
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>1570548</v>
+        <v>3110043</v>
       </c>
     </row>
     <row r="40">
@@ -1727,11 +1727,11 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1081</v>
+        <v>1501</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ADVOCACIA GERAL DO ESTADO</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -1747,31 +1747,31 @@
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>45000</v>
+        <v>1570548</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4381</v>
+        <v>4031</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
+          <t>FUNDO ESPECIAL DO PODER JUDICIÁRIO DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1251</v>
+        <v>1081</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
+          <t>ADVOCACIA GERAL DO ESTADO</t>
         </is>
       </c>
       <c r="E41" t="n">
         <v>3</v>
       </c>
       <c r="F41" t="n">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
@@ -1780,31 +1780,31 @@
         <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>15000000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2011</v>
+        <v>4381</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1941</v>
+        <v>1251</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>EGE-SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E42" t="n">
         <v>3</v>
       </c>
       <c r="F42" t="n">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="G42" t="n">
         <v>2</v>
@@ -1813,7 +1813,7 @@
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>150000</v>
+        <v>15000000</v>
       </c>
     </row>
     <row r="43">
@@ -1826,11 +1826,11 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1501</v>
+        <v>1941</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>EGE-SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -1846,16 +1846,16 @@
         <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>6311890</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1011</v>
+        <v>2011</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
+          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1879,39 +1879,72 @@
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>104706</v>
+        <v>6311890</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
+        <v>1011</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1501</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="n">
+        <v>60</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>104706</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
         <v>4111</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>FUNDO DE FOMENTO E DESENVOLVIMENTO SOCIOECONÔMICO DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
-      <c r="C45" t="n">
+      <c r="C46" t="n">
         <v>1915</v>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>PARTICIPAÇÃO NO AUMENTO DO CAPITAL SOCIAL DE EMPRESAS</t>
         </is>
       </c>
-      <c r="E45" t="n">
+      <c r="E46" t="n">
         <v>5</v>
       </c>
-      <c r="F45" t="n">
+      <c r="F46" t="n">
         <v>61</v>
       </c>
-      <c r="G45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0</v>
-      </c>
-      <c r="I45" t="n">
+      <c r="G46" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
         <v>98000</v>
       </c>
     </row>

</xml_diff>